<commit_message>
Rebuild templates with consistent category/subcategory taxonomy matching PROFIT's actual data structure
</commit_message>
<xml_diff>
--- a/docs/templates/PnL_Cashflow_Template.xlsx
+++ b/docs/templates/PnL_Cashflow_Template.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="33">
   <si>
     <t xml:space="preserve">Cara guna template ini</t>
   </si>
@@ -30,31 +30,37 @@
     <t xml:space="preserve">1. Ada 2 tab: 'PnL' dan 'Cashflow'. Isi tab yang berkaitan.</t>
   </si>
   <si>
-    <t xml:space="preserve">2. Jangan tukar nama header (Category, Subcategory, Amount) atau susunan column.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3. Padam baris contoh (bergaris kuning) sebelum upload data sebenar.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4. Amount: guna nombor positif untuk cash-in/revenue, negatif untuk cash-out/expense.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5. Subcategory boleh kosongkan jika tak perlu breakdown lanjut.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">6. Bila upload dalam app, pilih statement type (PnL/Cashflow) yang sepadan dengan tab.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">7. Simpan sebagai .xlsx atau export tab berkenaan sebagai .csv sebelum upload.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PnL Template — isi bermula dari baris 5. JANGAN tukar nama column (Category, Subcategory, Amount).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Category = kategori utama (cth: Revenue, COGS, Opex). Subcategory = butiran (optional, boleh kosongkan). Amount = nilai dalam RM (positif untuk masuk, negatif untuk keluar).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Padam baris contoh (bergaris kuning) sebelum upload, atau tulis ganti dengan data sebenar.</t>
+    <t xml:space="preserve">2. Category/Type dan Subcategory dalam template ni SAMA dengan yang app PROFIT guna — jangan tukar nama, supaya data automatik disusun betul.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3. Senarai Subcategory (Cost) standard: Direct Manpower, Project Allowance, Travel &amp; Accommodations, Vehicle Leasing / Cost, Equipment &amp; Hardware, Permit &amp; Regulatory, Other Direct Project Cost, Salary, Shared Service.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4. Boleh tambah Subcategory baru kalau perlu — app akan terima category/subcategory baru secara automatik.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5. Guna template ni kalau TAK perlu breakdown ikut bulan — satu total sahaja setiap item.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6. Untuk expense/Cash-Out, taip nombor POSITIF — app auto-tolak (negative) bila import.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7. Padam baris contoh (bergaris hijau) sebelum isi data sebenar.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8. Nak breakdown ikut bulan? Guna template 'Monthly' sebaliknya.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bila upload dalam app, pilih statement type (PnL/Cashflow) yang sepadan dengan tab yang diisi.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PnL Template (Flat) — isi bermula dari baris 5. Guna ni kalau TAK perlu breakdown ikut bulan (satu total sahaja per item).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Category = 'Revenue' atau 'Expenses'. Subcategory = item spesifik (sama senarai macam dalam app PROFIT — rujuk contoh di bawah).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Amount: untuk Expenses/expense, taip nombor POSITIF — app auto-tolak ikut Category. Padam baris contoh (bergaris hijau) sebelum isi data sebenar.</t>
   </si>
   <si>
     <t xml:space="preserve">Category</t>
@@ -69,34 +75,52 @@
     <t xml:space="preserve">Revenue</t>
   </si>
   <si>
-    <t xml:space="preserve">Project Billing</t>
-  </si>
-  <si>
-    <t xml:space="preserve">COGS</t>
+    <t xml:space="preserve">Client Payment</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Expenses</t>
   </si>
   <si>
     <t xml:space="preserve">Direct Manpower</t>
   </si>
   <si>
-    <t xml:space="preserve">Opex</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Software &amp; Licenses</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cashflow Template — isi bermula dari baris 5. JANGAN tukar nama column (Category, Subcategory, Amount).</t>
+    <t xml:space="preserve">Project Allowance</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Travel &amp; Accommodations</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vehicle Leasing / Cost</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Equipment &amp; Hardware</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Permit &amp; Regulatory</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Other Direct Project Cost</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Salary</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Shared Service</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cashflow Template (Flat) — isi bermula dari baris 5. Guna ni kalau TAK perlu breakdown ikut bulan (satu total sahaja per item).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Category = 'Cash-In' atau 'Cash-Out'. Subcategory = item spesifik (sama senarai macam dalam app PROFIT — rujuk contoh di bawah).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Amount: untuk Cash-Out/expense, taip nombor POSITIF — app auto-tolak ikut Category. Padam baris contoh (bergaris hijau) sebelum isi data sebenar.</t>
   </si>
   <si>
     <t xml:space="preserve">Cash-In</t>
   </si>
   <si>
-    <t xml:space="preserve">Client Payment</t>
-  </si>
-  <si>
     <t xml:space="preserve">Cash-Out</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Vehicle Cost</t>
   </si>
 </sst>
 </file>
@@ -133,14 +157,14 @@
     <font>
       <b val="true"/>
       <sz val="14"/>
-      <color rgb="FF1C2321"/>
+      <color rgb="FF101A2C"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FF1C2321"/>
+      <color rgb="FF101A2C"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
@@ -148,7 +172,7 @@
     <font>
       <b val="true"/>
       <sz val="11"/>
-      <color rgb="FF1C2321"/>
+      <color rgb="FF101A2C"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
@@ -156,29 +180,29 @@
     <font>
       <i val="true"/>
       <sz val="10"/>
-      <color rgb="FF8A8578"/>
+      <color rgb="FF6B6A63"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
     </font>
     <font>
       <b val="true"/>
-      <sz val="11"/>
-      <color rgb="FFF7F5F0"/>
+      <sz val="10.5"/>
+      <color rgb="FFFFFFFF"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
     </font>
     <font>
       <i val="true"/>
-      <sz val="11"/>
-      <color rgb="FF7A5E14"/>
+      <sz val="10.5"/>
+      <color rgb="FF2F8F86"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
     </font>
     <font>
-      <sz val="11"/>
+      <sz val="10.5"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
@@ -193,14 +217,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF1C2321"/>
-        <bgColor rgb="FF333300"/>
+        <fgColor rgb="FF101A2C"/>
+        <bgColor rgb="FF000000"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFF9E5"/>
-        <bgColor rgb="FFF7F5F0"/>
+        <fgColor rgb="FFE4F1EF"/>
+        <bgColor rgb="FFCCFFFF"/>
       </patternFill>
     </fill>
   </fills>
@@ -214,16 +238,16 @@
     </border>
     <border diagonalUp="false" diagonalDown="false">
       <left style="thin">
-        <color rgb="FFD8D3C6"/>
+        <color rgb="FFDCD8CB"/>
       </left>
       <right style="thin">
-        <color rgb="FFD8D3C6"/>
+        <color rgb="FFDCD8CB"/>
       </right>
       <top style="thin">
-        <color rgb="FFD8D3C6"/>
+        <color rgb="FFDCD8CB"/>
       </top>
       <bottom style="thin">
-        <color rgb="FFD8D3C6"/>
+        <color rgb="FFDCD8CB"/>
       </bottom>
       <diagonal/>
     </border>
@@ -310,7 +334,7 @@
   <colors>
     <indexedColors>
       <rgbColor rgb="FF000000"/>
-      <rgbColor rgb="FFF7F5F0"/>
+      <rgbColor rgb="FFFFFFFF"/>
       <rgbColor rgb="FFFF0000"/>
       <rgbColor rgb="FF00FF00"/>
       <rgbColor rgb="FF0000FF"/>
@@ -320,19 +344,19 @@
       <rgbColor rgb="FF800000"/>
       <rgbColor rgb="FF008000"/>
       <rgbColor rgb="FF000080"/>
-      <rgbColor rgb="FF7A5E14"/>
+      <rgbColor rgb="FF808000"/>
       <rgbColor rgb="FF800080"/>
       <rgbColor rgb="FF008080"/>
-      <rgbColor rgb="FFD8D3C6"/>
-      <rgbColor rgb="FF8A8578"/>
+      <rgbColor rgb="FFC0C0C0"/>
+      <rgbColor rgb="FF808080"/>
       <rgbColor rgb="FF9999FF"/>
       <rgbColor rgb="FF993366"/>
-      <rgbColor rgb="FFFFF9E5"/>
-      <rgbColor rgb="FFCCFFFF"/>
+      <rgbColor rgb="FFFFFFCC"/>
+      <rgbColor rgb="FFE4F1EF"/>
       <rgbColor rgb="FF660066"/>
       <rgbColor rgb="FFFF8080"/>
       <rgbColor rgb="FF0066CC"/>
-      <rgbColor rgb="FFCCCCFF"/>
+      <rgbColor rgb="FFDCD8CB"/>
       <rgbColor rgb="FF000080"/>
       <rgbColor rgb="FFFF00FF"/>
       <rgbColor rgb="FFFFFF00"/>
@@ -355,16 +379,16 @@
       <rgbColor rgb="FFFFCC00"/>
       <rgbColor rgb="FFFF9900"/>
       <rgbColor rgb="FFFF6600"/>
-      <rgbColor rgb="FF666699"/>
+      <rgbColor rgb="FF6B6A63"/>
       <rgbColor rgb="FF969696"/>
       <rgbColor rgb="FF003366"/>
-      <rgbColor rgb="FF339966"/>
-      <rgbColor rgb="FF003300"/>
+      <rgbColor rgb="FF2F8F86"/>
+      <rgbColor rgb="FF101A2C"/>
       <rgbColor rgb="FF333300"/>
       <rgbColor rgb="FF993300"/>
       <rgbColor rgb="FF993366"/>
       <rgbColor rgb="FF333399"/>
-      <rgbColor rgb="FF1C2321"/>
+      <rgbColor rgb="FF333333"/>
     </indexedColors>
   </colors>
 </styleSheet>
@@ -550,10 +574,10 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:A9"/>
+  <dimension ref="A1:A12"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="90"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="95"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -569,17 +593,17 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
         <v>4</v>
       </c>
@@ -597,6 +621,19 @@
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
         <v>7</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="2"/>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="2" t="s">
+        <v>9</v>
       </c>
     </row>
   </sheetData>
@@ -618,48 +655,49 @@
   <dimension ref="A1:C23"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="1" style="0" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="28"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="16"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="3" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B1" s="3"/>
       <c r="C1" s="3"/>
     </row>
     <row r="2" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="4" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="B2" s="4"/>
       <c r="C2" s="4"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="5" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B3" s="5"/>
       <c r="C3" s="5"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="7" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="C6" s="8" t="n">
         <v>150000</v>
@@ -667,13 +705,13 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="7" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="C7" s="8" t="n">
-        <v>-62000</v>
+        <v>25000</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -681,45 +719,77 @@
         <v>18</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C8" s="8" t="n">
-        <v>-3200</v>
+        <v>25000</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="9"/>
-      <c r="B9" s="9"/>
-      <c r="C9" s="10"/>
+      <c r="A9" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="B9" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="C9" s="8" t="n">
+        <v>25000</v>
+      </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="9"/>
-      <c r="B10" s="9"/>
-      <c r="C10" s="10"/>
+      <c r="A10" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="B10" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="C10" s="8" t="n">
+        <v>25000</v>
+      </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="9"/>
-      <c r="B11" s="9"/>
+      <c r="A11" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="B11" s="9" t="s">
+        <v>23</v>
+      </c>
       <c r="C11" s="10"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="9"/>
-      <c r="B12" s="9"/>
+      <c r="A12" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="B12" s="9" t="s">
+        <v>24</v>
+      </c>
       <c r="C12" s="10"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="9"/>
-      <c r="B13" s="9"/>
+      <c r="A13" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="B13" s="9" t="s">
+        <v>25</v>
+      </c>
       <c r="C13" s="10"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="9"/>
-      <c r="B14" s="9"/>
+      <c r="A14" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="B14" s="9" t="s">
+        <v>26</v>
+      </c>
       <c r="C14" s="10"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="9"/>
-      <c r="B15" s="9"/>
+      <c r="A15" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="B15" s="9" t="s">
+        <v>27</v>
+      </c>
       <c r="C15" s="10"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -786,48 +856,49 @@
   <dimension ref="A1:C23"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="1" style="0" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="28"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="16"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="3" t="s">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="B1" s="3"/>
       <c r="C1" s="3"/>
     </row>
     <row r="2" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="4" t="s">
-        <v>9</v>
+        <v>29</v>
       </c>
       <c r="B2" s="4"/>
       <c r="C2" s="4"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="5" t="s">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="B3" s="5"/>
       <c r="C3" s="5"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="7" t="s">
-        <v>21</v>
+        <v>31</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="C6" s="8" t="n">
         <v>150000</v>
@@ -835,59 +906,91 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="7" t="s">
-        <v>23</v>
+        <v>32</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="C7" s="8" t="n">
-        <v>-62000</v>
+        <v>25000</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="B8" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="C8" s="8" t="n">
+        <v>25000</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="B9" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="C9" s="8" t="n">
+        <v>25000</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="B10" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="C10" s="8" t="n">
+        <v>25000</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="9" t="s">
+        <v>32</v>
+      </c>
+      <c r="B11" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="B8" s="7" t="s">
+      <c r="C11" s="10"/>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="9" t="s">
+        <v>32</v>
+      </c>
+      <c r="B12" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="C8" s="8" t="n">
-        <v>-2350.6</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="9"/>
-      <c r="B9" s="9"/>
-      <c r="C9" s="10"/>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="9"/>
-      <c r="B10" s="9"/>
-      <c r="C10" s="10"/>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="9"/>
-      <c r="B11" s="9"/>
-      <c r="C11" s="10"/>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="9"/>
-      <c r="B12" s="9"/>
       <c r="C12" s="10"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="9"/>
-      <c r="B13" s="9"/>
+      <c r="A13" s="9" t="s">
+        <v>32</v>
+      </c>
+      <c r="B13" s="9" t="s">
+        <v>25</v>
+      </c>
       <c r="C13" s="10"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="9"/>
-      <c r="B14" s="9"/>
+      <c r="A14" s="9" t="s">
+        <v>32</v>
+      </c>
+      <c r="B14" s="9" t="s">
+        <v>26</v>
+      </c>
       <c r="C14" s="10"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="9"/>
-      <c r="B15" s="9"/>
+      <c r="A15" s="9" t="s">
+        <v>32</v>
+      </c>
+      <c r="B15" s="9" t="s">
+        <v>27</v>
+      </c>
       <c r="C15" s="10"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Make Month mandatory across app and templates; fix monthly template import to preserve per-month data instead of collapsing to totals
</commit_message>
<xml_diff>
--- a/docs/templates/PnL_Cashflow_Template.xlsx
+++ b/docs/templates/PnL_Cashflow_Template.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="38">
   <si>
     <t xml:space="preserve">Cara guna template ini</t>
   </si>
@@ -39,28 +39,34 @@
     <t xml:space="preserve">4. Boleh tambah Subcategory baru kalau perlu — app akan terima category/subcategory baru secara automatik.</t>
   </si>
   <si>
-    <t xml:space="preserve">5. Guna template ni kalau TAK perlu breakdown ikut bulan — satu total sahaja setiap item.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">6. Untuk expense/Cash-Out, taip nombor POSITIF — app auto-tolak (negative) bila import.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">7. Padam baris contoh (bergaris hijau) sebelum isi data sebenar.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">8. Nak breakdown ikut bulan? Guna template 'Monthly' sebaliknya.</t>
+    <t xml:space="preserve">5. MONTH ADALAH WAJIB — PROFIT perlukan bulan pada SETIAP baris data untuk Grid view, Forecast, dan laporan trend bulanan berfungsi. Data tanpa bulan akan DITOLAK semasa upload.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6. Column Month: format 'MMM-YY' (cth: Jan-26) atau 'YYYY-MM' (cth: 2026-01).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7. Untuk item yang sama tapi bulan berbeza, taip baris BERASINGAN untuk setiap bulan (bukan satu baris untuk semua bulan).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8. Untuk expense/Cash-Out, taip nombor POSITIF — app auto-tolak (negative) bila import.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">9. Padam baris contoh (bergaris hijau) sebelum isi data sebenar.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10. Nak isi banyak bulan untuk satu item sekali gus? Guna template 'Monthly' sebaliknya (lagi cepat).</t>
   </si>
   <si>
     <t xml:space="preserve">Bila upload dalam app, pilih statement type (PnL/Cashflow) yang sepadan dengan tab yang diisi.</t>
   </si>
   <si>
-    <t xml:space="preserve">PnL Template (Flat) — isi bermula dari baris 5. Guna ni kalau TAK perlu breakdown ikut bulan (satu total sahaja per item).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Category = 'Revenue' atau 'Expenses'. Subcategory = item spesifik (sama senarai macam dalam app PROFIT — rujuk contoh di bawah).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Amount: untuk Expenses/expense, taip nombor POSITIF — app auto-tolak ikut Category. Padam baris contoh (bergaris hijau) sebelum isi data sebenar.</t>
+    <t xml:space="preserve">PnL Template (Flat) — isi bermula dari baris 5. Format 'long list': satu baris = satu item untuk SATU bulan.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Category = 'Revenue' atau 'Expenses'. Subcategory = item spesifik. Month WAJIB diisi — format 'MMM-YY' (contoh: Jan-26) atau 'YYYY-MM' (contoh: 2026-01).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Amount: untuk Expenses/expense, taip nombor POSITIF — app auto-tolak ikut Category. Ada dua baris untuk bulan berbeza untuk item yang sama? Taip DUA baris berasingan (satu setiap bulan).</t>
   </si>
   <si>
     <t xml:space="preserve">Category</t>
@@ -69,6 +75,9 @@
     <t xml:space="preserve">Subcategory</t>
   </si>
   <si>
+    <t xml:space="preserve">Month</t>
+  </si>
+  <si>
     <t xml:space="preserve">Amount</t>
   </si>
   <si>
@@ -78,6 +87,12 @@
     <t xml:space="preserve">Client Payment</t>
   </si>
   <si>
+    <t xml:space="preserve">Jan-26</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Feb-26</t>
+  </si>
+  <si>
     <t xml:space="preserve">Expenses</t>
   </si>
   <si>
@@ -108,13 +123,13 @@
     <t xml:space="preserve">Shared Service</t>
   </si>
   <si>
-    <t xml:space="preserve">Cashflow Template (Flat) — isi bermula dari baris 5. Guna ni kalau TAK perlu breakdown ikut bulan (satu total sahaja per item).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Category = 'Cash-In' atau 'Cash-Out'. Subcategory = item spesifik (sama senarai macam dalam app PROFIT — rujuk contoh di bawah).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Amount: untuk Cash-Out/expense, taip nombor POSITIF — app auto-tolak ikut Category. Padam baris contoh (bergaris hijau) sebelum isi data sebenar.</t>
+    <t xml:space="preserve">Cashflow Template (Flat) — isi bermula dari baris 5. Format 'long list': satu baris = satu item untuk SATU bulan.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Category = 'Cash-In' atau 'Cash-Out'. Subcategory = item spesifik. Month WAJIB diisi — format 'MMM-YY' (contoh: Jan-26) atau 'YYYY-MM' (contoh: 2026-01).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Amount: untuk Cash-Out/expense, taip nombor POSITIF — app auto-tolak ikut Category. Ada dua baris untuk bulan berbeza untuk item yang sama? Taip DUA baris berasingan (satu setiap bulan).</t>
   </si>
   <si>
     <t xml:space="preserve">Cash-In</t>
@@ -277,7 +292,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -287,6 +302,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -574,7 +593,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:A12"/>
+  <dimension ref="A1:A14"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="95"/>
@@ -608,8 +627,8 @@
         <v>4</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="2" t="s">
+    <row r="7" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="3" t="s">
         <v>5</v>
       </c>
     </row>
@@ -618,7 +637,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
         <v>7</v>
       </c>
@@ -629,11 +648,21 @@
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="2"/>
+      <c r="A11" s="2" t="s">
+        <v>9</v>
+      </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>9</v>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="2"/>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="2" t="s">
+        <v>11</v>
       </c>
     </row>
   </sheetData>
@@ -652,191 +681,247 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C23"/>
+  <dimension ref="A1:D26"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="26"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="28"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="1" style="0" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="16"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="B1" s="3"/>
-      <c r="C1" s="3"/>
+      <c r="A1" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B1" s="4"/>
+      <c r="C1" s="4"/>
+      <c r="D1" s="4"/>
     </row>
     <row r="2" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="B2" s="4"/>
-      <c r="C2" s="4"/>
+      <c r="A2" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="B2" s="5"/>
+      <c r="C2" s="5"/>
+      <c r="D2" s="5"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="B3" s="5"/>
-      <c r="C3" s="5"/>
+      <c r="A3" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="B3" s="6"/>
+      <c r="C3" s="6"/>
+      <c r="D3" s="6"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="B5" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="C5" s="6" t="s">
+      <c r="A5" s="7" t="s">
         <v>15</v>
       </c>
+      <c r="B5" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="C5" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="D5" s="7" t="s">
+        <v>18</v>
+      </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="B6" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="C6" s="8" t="n">
+      <c r="A6" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="B6" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="C6" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="D6" s="9" t="n">
         <v>150000</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="7" t="s">
-        <v>18</v>
-      </c>
-      <c r="B7" s="7" t="s">
+      <c r="A7" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="C7" s="8" t="n">
+      <c r="B7" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="C7" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="D7" s="9" t="n">
+        <v>90000</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="B8" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="C8" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="D8" s="9" t="n">
         <v>25000</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="7" t="s">
-        <v>18</v>
-      </c>
-      <c r="B8" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="C8" s="8" t="n">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="B9" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="C9" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="D9" s="9" t="n">
         <v>25000</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="7" t="s">
-        <v>18</v>
-      </c>
-      <c r="B9" s="7" t="s">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="B10" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="C10" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="C9" s="8" t="n">
+      <c r="D10" s="9" t="n">
         <v>25000</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="7" t="s">
-        <v>18</v>
-      </c>
-      <c r="B10" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="C10" s="8" t="n">
-        <v>25000</v>
-      </c>
-    </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="9" t="s">
-        <v>18</v>
-      </c>
-      <c r="B11" s="9" t="s">
+      <c r="A11" s="10" t="s">
         <v>23</v>
       </c>
+      <c r="B11" s="10" t="s">
+        <v>27</v>
+      </c>
       <c r="C11" s="10"/>
+      <c r="D11" s="11"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="9" t="s">
-        <v>18</v>
-      </c>
-      <c r="B12" s="9" t="s">
-        <v>24</v>
+      <c r="A12" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="B12" s="10" t="s">
+        <v>28</v>
       </c>
       <c r="C12" s="10"/>
+      <c r="D12" s="11"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="9" t="s">
-        <v>18</v>
-      </c>
-      <c r="B13" s="9" t="s">
-        <v>25</v>
+      <c r="A13" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="B13" s="10" t="s">
+        <v>29</v>
       </c>
       <c r="C13" s="10"/>
+      <c r="D13" s="11"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="9" t="s">
-        <v>18</v>
-      </c>
-      <c r="B14" s="9" t="s">
-        <v>26</v>
+      <c r="A14" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="B14" s="10" t="s">
+        <v>30</v>
       </c>
       <c r="C14" s="10"/>
+      <c r="D14" s="11"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="9" t="s">
-        <v>18</v>
-      </c>
-      <c r="B15" s="9" t="s">
-        <v>27</v>
+      <c r="A15" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="B15" s="10" t="s">
+        <v>31</v>
       </c>
       <c r="C15" s="10"/>
+      <c r="D15" s="11"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="9"/>
-      <c r="B16" s="9"/>
+      <c r="A16" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="B16" s="10" t="s">
+        <v>32</v>
+      </c>
       <c r="C16" s="10"/>
+      <c r="D16" s="11"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="9"/>
-      <c r="B17" s="9"/>
+      <c r="A17" s="10"/>
+      <c r="B17" s="10"/>
       <c r="C17" s="10"/>
+      <c r="D17" s="11"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="9"/>
-      <c r="B18" s="9"/>
+      <c r="A18" s="10"/>
+      <c r="B18" s="10"/>
       <c r="C18" s="10"/>
+      <c r="D18" s="11"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="9"/>
-      <c r="B19" s="9"/>
+      <c r="A19" s="10"/>
+      <c r="B19" s="10"/>
       <c r="C19" s="10"/>
+      <c r="D19" s="11"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="9"/>
-      <c r="B20" s="9"/>
+      <c r="A20" s="10"/>
+      <c r="B20" s="10"/>
       <c r="C20" s="10"/>
+      <c r="D20" s="11"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="9"/>
-      <c r="B21" s="9"/>
+      <c r="A21" s="10"/>
+      <c r="B21" s="10"/>
       <c r="C21" s="10"/>
+      <c r="D21" s="11"/>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="9"/>
-      <c r="B22" s="9"/>
+      <c r="A22" s="10"/>
+      <c r="B22" s="10"/>
       <c r="C22" s="10"/>
+      <c r="D22" s="11"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="9"/>
-      <c r="B23" s="9"/>
+      <c r="A23" s="10"/>
+      <c r="B23" s="10"/>
       <c r="C23" s="10"/>
+      <c r="D23" s="11"/>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="10"/>
+      <c r="B24" s="10"/>
+      <c r="C24" s="10"/>
+      <c r="D24" s="11"/>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="10"/>
+      <c r="B25" s="10"/>
+      <c r="C25" s="10"/>
+      <c r="D25" s="11"/>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="10"/>
+      <c r="B26" s="10"/>
+      <c r="C26" s="10"/>
+      <c r="D26" s="11"/>
     </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="A1:C1"/>
-    <mergeCell ref="A2:C2"/>
-    <mergeCell ref="A3:C3"/>
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A2:D2"/>
+    <mergeCell ref="A3:D3"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -853,191 +938,247 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C23"/>
+  <dimension ref="A1:D26"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="26"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="28"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="1" style="0" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="16"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="B1" s="4"/>
+      <c r="C1" s="4"/>
+      <c r="D1" s="4"/>
+    </row>
+    <row r="2" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="B2" s="5"/>
+      <c r="C2" s="5"/>
+      <c r="D2" s="5"/>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="B3" s="6"/>
+      <c r="C3" s="6"/>
+      <c r="D3" s="6"/>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="B5" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="C5" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="D5" s="7" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="B6" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="C6" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="D6" s="9" t="n">
+        <v>150000</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="B7" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="C7" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="D7" s="9" t="n">
+        <v>90000</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="B8" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="C8" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="D8" s="9" t="n">
+        <v>25000</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="B9" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="C9" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="D9" s="9" t="n">
+        <v>25000</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="B10" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="C10" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="D10" s="9" t="n">
+        <v>25000</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="10" t="s">
+        <v>37</v>
+      </c>
+      <c r="B11" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="C11" s="10"/>
+      <c r="D11" s="11"/>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="10" t="s">
+        <v>37</v>
+      </c>
+      <c r="B12" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="B1" s="3"/>
-      <c r="C1" s="3"/>
-    </row>
-    <row r="2" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="4" t="s">
+      <c r="C12" s="10"/>
+      <c r="D12" s="11"/>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="10" t="s">
+        <v>37</v>
+      </c>
+      <c r="B13" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="B2" s="4"/>
-      <c r="C2" s="4"/>
-    </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="5" t="s">
+      <c r="C13" s="10"/>
+      <c r="D13" s="11"/>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="10" t="s">
+        <v>37</v>
+      </c>
+      <c r="B14" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="B3" s="5"/>
-      <c r="C3" s="5"/>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="B5" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="C5" s="6" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="7" t="s">
+      <c r="C14" s="10"/>
+      <c r="D14" s="11"/>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="10" t="s">
+        <v>37</v>
+      </c>
+      <c r="B15" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="B6" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="C6" s="8" t="n">
-        <v>150000</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="7" t="s">
+      <c r="C15" s="10"/>
+      <c r="D15" s="11"/>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="10" t="s">
+        <v>37</v>
+      </c>
+      <c r="B16" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="B7" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="C7" s="8" t="n">
-        <v>25000</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="7" t="s">
-        <v>32</v>
-      </c>
-      <c r="B8" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="C8" s="8" t="n">
-        <v>25000</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="7" t="s">
-        <v>32</v>
-      </c>
-      <c r="B9" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="C9" s="8" t="n">
-        <v>25000</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="7" t="s">
-        <v>32</v>
-      </c>
-      <c r="B10" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="C10" s="8" t="n">
-        <v>25000</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="B11" s="9" t="s">
-        <v>23</v>
-      </c>
-      <c r="C11" s="10"/>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="B12" s="9" t="s">
-        <v>24</v>
-      </c>
-      <c r="C12" s="10"/>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="B13" s="9" t="s">
-        <v>25</v>
-      </c>
-      <c r="C13" s="10"/>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="B14" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="C14" s="10"/>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="B15" s="9" t="s">
-        <v>27</v>
-      </c>
-      <c r="C15" s="10"/>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="9"/>
-      <c r="B16" s="9"/>
       <c r="C16" s="10"/>
+      <c r="D16" s="11"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="9"/>
-      <c r="B17" s="9"/>
+      <c r="A17" s="10"/>
+      <c r="B17" s="10"/>
       <c r="C17" s="10"/>
+      <c r="D17" s="11"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="9"/>
-      <c r="B18" s="9"/>
+      <c r="A18" s="10"/>
+      <c r="B18" s="10"/>
       <c r="C18" s="10"/>
+      <c r="D18" s="11"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="9"/>
-      <c r="B19" s="9"/>
+      <c r="A19" s="10"/>
+      <c r="B19" s="10"/>
       <c r="C19" s="10"/>
+      <c r="D19" s="11"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="9"/>
-      <c r="B20" s="9"/>
+      <c r="A20" s="10"/>
+      <c r="B20" s="10"/>
       <c r="C20" s="10"/>
+      <c r="D20" s="11"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="9"/>
-      <c r="B21" s="9"/>
+      <c r="A21" s="10"/>
+      <c r="B21" s="10"/>
       <c r="C21" s="10"/>
+      <c r="D21" s="11"/>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="9"/>
-      <c r="B22" s="9"/>
+      <c r="A22" s="10"/>
+      <c r="B22" s="10"/>
       <c r="C22" s="10"/>
+      <c r="D22" s="11"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="9"/>
-      <c r="B23" s="9"/>
+      <c r="A23" s="10"/>
+      <c r="B23" s="10"/>
       <c r="C23" s="10"/>
+      <c r="D23" s="11"/>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="10"/>
+      <c r="B24" s="10"/>
+      <c r="C24" s="10"/>
+      <c r="D24" s="11"/>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="10"/>
+      <c r="B25" s="10"/>
+      <c r="C25" s="10"/>
+      <c r="D25" s="11"/>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="10"/>
+      <c r="B26" s="10"/>
+      <c r="C26" s="10"/>
+      <c r="D26" s="11"/>
     </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="A1:C1"/>
-    <mergeCell ref="A2:C2"/>
-    <mergeCell ref="A3:C3"/>
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A2:D2"/>
+    <mergeCell ref="A3:D3"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
Translate Excel templates (How To Use tab + all instructions) to English, matching app-wide English-only rule
</commit_message>
<xml_diff>
--- a/docs/templates/PnL_Cashflow_Template.xlsx
+++ b/docs/templates/PnL_Cashflow_Template.xlsx
@@ -8,7 +8,7 @@
     <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="Cara Guna" sheetId="1" state="visible" r:id="rId3"/>
+    <sheet name="How To Use" sheetId="1" state="visible" r:id="rId3"/>
     <sheet name="PnL" sheetId="2" state="visible" r:id="rId4"/>
     <sheet name="Cashflow" sheetId="3" state="visible" r:id="rId5"/>
   </sheets>
@@ -24,49 +24,49 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="38">
   <si>
-    <t xml:space="preserve">Cara guna template ini</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Ada 2 tab: 'PnL' dan 'Cashflow'. Isi tab yang berkaitan.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2. Category/Type dan Subcategory dalam template ni SAMA dengan yang app PROFIT guna — jangan tukar nama, supaya data automatik disusun betul.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3. Senarai Subcategory (Cost) standard: Direct Manpower, Project Allowance, Travel &amp; Accommodations, Vehicle Leasing / Cost, Equipment &amp; Hardware, Permit &amp; Regulatory, Other Direct Project Cost, Salary, Shared Service.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4. Boleh tambah Subcategory baru kalau perlu — app akan terima category/subcategory baru secara automatik.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5. MONTH ADALAH WAJIB — PROFIT perlukan bulan pada SETIAP baris data untuk Grid view, Forecast, dan laporan trend bulanan berfungsi. Data tanpa bulan akan DITOLAK semasa upload.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">6. Column Month: format 'MMM-YY' (cth: Jan-26) atau 'YYYY-MM' (cth: 2026-01).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">7. Untuk item yang sama tapi bulan berbeza, taip baris BERASINGAN untuk setiap bulan (bukan satu baris untuk semua bulan).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">8. Untuk expense/Cash-Out, taip nombor POSITIF — app auto-tolak (negative) bila import.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">9. Padam baris contoh (bergaris hijau) sebelum isi data sebenar.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">10. Nak isi banyak bulan untuk satu item sekali gus? Guna template 'Monthly' sebaliknya (lagi cepat).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bila upload dalam app, pilih statement type (PnL/Cashflow) yang sepadan dengan tab yang diisi.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PnL Template (Flat) — isi bermula dari baris 5. Format 'long list': satu baris = satu item untuk SATU bulan.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Category = 'Revenue' atau 'Expenses'. Subcategory = item spesifik. Month WAJIB diisi — format 'MMM-YY' (contoh: Jan-26) atau 'YYYY-MM' (contoh: 2026-01).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Amount: untuk Expenses/expense, taip nombor POSITIF — app auto-tolak ikut Category. Ada dua baris untuk bulan berbeza untuk item yang sama? Taip DUA baris berasingan (satu setiap bulan).</t>
+    <t xml:space="preserve">How to use this template</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. There are 2 tabs: 'PnL' and 'Cashflow'. Fill in the relevant tab.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2. The Category/Type and Subcategory names in this template match exactly what PROFIT uses — do not rename them, so data is sorted correctly automatically.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3. Standard cost Subcategory list: Direct Manpower, Project Allowance, Travel &amp; Accommodations, Vehicle Leasing / Cost, Equipment &amp; Hardware, Permit &amp; Regulatory, Other Direct Project Cost, Salary, Shared Service.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4. You can add new Subcategories if needed — the app will accept new category/subcategory names automatically.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5. MONTH IS REQUIRED — PROFIT needs a month on every row of data for Grid view, Forecast, and monthly trend reporting to work. Data without a month will be REJECTED on upload.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6. Month column: format 'MMM-YY' (e.g. Jan-26) or 'YYYY-MM' (e.g. 2026-01).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7. For the same item across different months, add a SEPARATE row for each month (not one row covering all months).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8. For expenses/Cash-Out, type POSITIVE numbers — the app auto-flips the sign (negative) on import.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">9. Delete the example rows (highlighted green) before entering real data.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10. Need to fill many months for one item at once? Use the 'Monthly' template instead (faster).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">When uploading in the app, select the statement type (PnL/Cashflow) that matches the tab you filled in.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PnL Template (Flat) — start filling from row 5. Long-list format: one row = one item for ONE month.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Category = 'Revenue' or 'Expenses'. Subcategory = the specific item. Month is REQUIRED — format 'MMM-YY' (e.g. Jan-26) or 'YYYY-MM' (e.g. 2026-01).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Amount: for Expenses/expenses, type POSITIVE numbers — the app auto-flips the sign based on Category. Same item, different month? Add a SEPARATE row for each month.</t>
   </si>
   <si>
     <t xml:space="preserve">Category</t>
@@ -123,13 +123,13 @@
     <t xml:space="preserve">Shared Service</t>
   </si>
   <si>
-    <t xml:space="preserve">Cashflow Template (Flat) — isi bermula dari baris 5. Format 'long list': satu baris = satu item untuk SATU bulan.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Category = 'Cash-In' atau 'Cash-Out'. Subcategory = item spesifik. Month WAJIB diisi — format 'MMM-YY' (contoh: Jan-26) atau 'YYYY-MM' (contoh: 2026-01).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Amount: untuk Cash-Out/expense, taip nombor POSITIF — app auto-tolak ikut Category. Ada dua baris untuk bulan berbeza untuk item yang sama? Taip DUA baris berasingan (satu setiap bulan).</t>
+    <t xml:space="preserve">Cashflow Template (Flat) — start filling from row 5. Long-list format: one row = one item for ONE month.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Category = 'Cash-In' or 'Cash-Out'. Subcategory = the specific item. Month is REQUIRED — format 'MMM-YY' (e.g. Jan-26) or 'YYYY-MM' (e.g. 2026-01).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Amount: for Cash-Out/expenses, type POSITIVE numbers — the app auto-flips the sign based on Category. Same item, different month? Add a SEPARATE row for each month.</t>
   </si>
   <si>
     <t xml:space="preserve">Cash-In</t>
@@ -642,7 +642,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
         <v>8</v>
       </c>
@@ -660,7 +660,7 @@
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2"/>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="14" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="s">
         <v>11</v>
       </c>

</xml_diff>